<commit_message>
Update cleaned delivery data in Cleaned_delivery.xlsx
</commit_message>
<xml_diff>
--- a/Aug_2/Cleaned_delivery.xlsx
+++ b/Aug_2/Cleaned_delivery.xlsx
@@ -232,70 +232,70 @@
     <t>212-555-0100</t>
   </si>
   <si>
-    <t>Burger, Fries, Coke</t>
-  </si>
-  <si>
-    <t>Pizza, Garlic Bread, Soda</t>
-  </si>
-  <si>
-    <t>Salad, Water</t>
-  </si>
-  <si>
-    <t>Tacos, Tacos, Chips</t>
-  </si>
-  <si>
-    <t>Sushi Roll, Miso Soup</t>
-  </si>
-  <si>
-    <t>Burger, Coke</t>
-  </si>
-  <si>
-    <t>Pad Thai, Spring Rolls, Thai Tea</t>
-  </si>
-  <si>
-    <t>Wings, Fries</t>
-  </si>
-  <si>
-    <t>Ramen, Gyoza, Green Tea</t>
-  </si>
-  <si>
-    <t>Curry, Naan, Rice</t>
-  </si>
-  <si>
-    <t>Falafel Wrap, Hummus</t>
-  </si>
-  <si>
-    <t>Steak, Mashed Potatoes, Wine</t>
-  </si>
-  <si>
-    <t>Dosa, Chutney, Chai</t>
-  </si>
-  <si>
-    <t>Burger, Onion Rings</t>
-  </si>
-  <si>
-    <t>Ceviche, Tostones</t>
-  </si>
-  <si>
-    <t>Pho, Spring Rolls</t>
-  </si>
-  <si>
-    <t>Biryani, Raita</t>
-  </si>
-  <si>
-    <t>Jollof Rice, Chicken, Plantains</t>
-  </si>
-  <si>
-    <t>Ramen, Gyoza</t>
-  </si>
-  <si>
-    <t>Jollof Rice, Suya</t>
-  </si>
-  <si>
-    <t>Bibimbap, Kimchi</t>
-  </si>
-  <si>
-    <t>Burger, Fries</t>
+    <t>B, u, r, g, e, r, ,,  , F, r, i, e, s, ,,  , C, o, k, e</t>
+  </si>
+  <si>
+    <t>P, i, z, z, a, ,,  , G, a, r, l, i, c,  , B, r, e, a, d, ,,  , S, o, d, a</t>
+  </si>
+  <si>
+    <t>S, a, l, a, d, ,,  , W, a, t, e, r</t>
+  </si>
+  <si>
+    <t>T, a, c, o, s, ,,  , T, a, c, o, s, ,,  , C, h, i, p, s</t>
+  </si>
+  <si>
+    <t>S, u, s, h, i,  , R, o, l, l, ,,  , M, i, s, o,  , S, o, u, p</t>
+  </si>
+  <si>
+    <t>B, u, r, g, e, r, ,,  , C, o, k, e</t>
+  </si>
+  <si>
+    <t>P, a, d,  , T, h, a, i, ,,  , S, p, r, i, n, g,  , R, o, l, l, s, ,,  , T, h, a, i,  , T, e, a</t>
+  </si>
+  <si>
+    <t>W, i, n, g, s, ,,  , F, r, i, e, s</t>
+  </si>
+  <si>
+    <t>R, a, m, e, n, ,,  , G, y, o, z, a, ,,  , G, r, e, e, n,  , T, e, a</t>
+  </si>
+  <si>
+    <t>C, u, r, r, y, ,,  , N, a, a, n, ,,  , R, i, c, e</t>
+  </si>
+  <si>
+    <t>F, a, l, a, f, e, l,  , W, r, a, p, ,,  , H, u, m, m, u, s</t>
+  </si>
+  <si>
+    <t>S, t, e, a, k, ,,  , M, a, s, h, e, d,  , P, o, t, a, t, o, e, s, ,,  , W, i, n, e</t>
+  </si>
+  <si>
+    <t>D, o, s, a, ,,  , C, h, u, t, n, e, y, ,,  , C, h, a, i</t>
+  </si>
+  <si>
+    <t>B, u, r, g, e, r, ,,  , O, n, i, o, n,  , R, i, n, g, s</t>
+  </si>
+  <si>
+    <t>C, e, v, i, c, h, e, ,,  , T, o, s, t, o, n, e, s</t>
+  </si>
+  <si>
+    <t>P, h, o, ,,  , S, p, r, i, n, g,  , R, o, l, l, s</t>
+  </si>
+  <si>
+    <t>B, i, r, y, a, n, i, ,,  , R, a, i, t, a</t>
+  </si>
+  <si>
+    <t>J, o, l, l, o, f,  , R, i, c, e, ,,  , C, h, i, c, k, e, n, ,,  , P, l, a, n, t, a, i, n, s</t>
+  </si>
+  <si>
+    <t>R, a, m, e, n, ,,  , G, y, o, z, a</t>
+  </si>
+  <si>
+    <t>J, o, l, l, o, f,  , R, i, c, e, ,,  , S, u, y, a</t>
+  </si>
+  <si>
+    <t>B, i, b, i, m, b, a, p, ,,  , K, i, m, c, h, i</t>
+  </si>
+  <si>
+    <t>B, u, r, g, e, r, ,,  , F, r, i, e, s</t>
   </si>
   <si>
     <t>Credit Card</t>

</xml_diff>